<commit_message>
fix error ca làm
</commit_message>
<xml_diff>
--- a/BE/ca_lam_xtep.xlsx
+++ b/BE/ca_lam_xtep.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ADMIN\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ADMIN\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0C6A6178-737A-48E8-A60F-9FCCE19EBA99}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1DEF6208-AEF7-4142-A89D-205814AA5D20}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28695" yWindow="0" windowWidth="16410" windowHeight="14145" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="2" r:id="rId1"/>
@@ -30,9 +30,6 @@
     <t>Cửa hàng</t>
   </si>
   <si>
-    <t>Royal City</t>
-  </si>
-  <si>
     <t>Vincom Việt Trì</t>
   </si>
   <si>
@@ -270,6 +267,9 @@
   <si>
     <t>7:30 - 15:30
 14:00 - 22:00</t>
+  </si>
+  <si>
+    <t>Royal</t>
   </si>
 </sst>
 </file>
@@ -620,319 +620,319 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
     <row r="2" spans="1:2" ht="45" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
-        <v>1</v>
+        <v>59</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="3" spans="1:2" ht="30" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="4" spans="1:2" ht="45" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="5" spans="1:2" ht="45" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="6" spans="1:2" ht="30" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
     <row r="7" spans="1:2" ht="90" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="8" spans="1:2" ht="60" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="9" spans="1:2" ht="90" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="10" spans="1:2" ht="120" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="11" spans="1:2" ht="45" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="12" spans="1:2" ht="45" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="13" spans="1:2" ht="45" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="14" spans="1:2" ht="120" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="15" spans="1:2" ht="45" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="16" spans="1:2" ht="45" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="17" spans="1:2" ht="45" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="18" spans="1:2" ht="45" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="19" spans="1:2" ht="90" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="20" spans="1:2" ht="45" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="21" spans="1:2" ht="45" x14ac:dyDescent="0.25">
       <c r="A21" s="1" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="22" spans="1:2" ht="45" x14ac:dyDescent="0.25">
       <c r="A22" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B22" s="3" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="23" spans="1:2" ht="30" x14ac:dyDescent="0.25">
       <c r="A23" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B23" s="3" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="24" spans="1:2" ht="30" x14ac:dyDescent="0.25">
       <c r="A24" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B24" s="3" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="25" spans="1:2" ht="120" x14ac:dyDescent="0.25">
       <c r="A25" s="1" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B25" s="3" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="26" spans="1:2" ht="90" x14ac:dyDescent="0.25">
       <c r="A26" s="1" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B26" s="3" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="27" spans="1:2" ht="45" x14ac:dyDescent="0.25">
       <c r="A27" s="1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B27" s="3" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="28" spans="1:2" ht="30" x14ac:dyDescent="0.25">
       <c r="A28" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B28" s="3" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="29" spans="1:2" ht="45" x14ac:dyDescent="0.25">
       <c r="A29" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B29" s="3" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="30" spans="1:2" ht="45" x14ac:dyDescent="0.25">
       <c r="A30" s="1" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B30" s="3" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="31" spans="1:2" ht="135" x14ac:dyDescent="0.25">
       <c r="A31" s="1" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B31" s="3" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="32" spans="1:2" ht="30" x14ac:dyDescent="0.25">
       <c r="A32" s="1" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B32" s="3" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="33" spans="1:2" ht="45" x14ac:dyDescent="0.25">
       <c r="A33" s="1" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B33" s="3" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="34" spans="1:2" ht="45" x14ac:dyDescent="0.25">
       <c r="A34" s="1" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B34" s="3" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="35" spans="1:2" ht="45" x14ac:dyDescent="0.25">
       <c r="A35" s="1" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B35" s="3" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="36" spans="1:2" ht="120" x14ac:dyDescent="0.25">
       <c r="A36" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B36" s="3" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="37" spans="1:2" ht="45" x14ac:dyDescent="0.25">
       <c r="A37" s="1" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B37" s="3" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="38" spans="1:2" ht="180" x14ac:dyDescent="0.25">
       <c r="A38" s="1" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B38" s="3" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="39" spans="1:2" ht="45" x14ac:dyDescent="0.25">
       <c r="A39" s="1" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B39" s="3" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
     <row r="40" spans="1:2" ht="45" x14ac:dyDescent="0.25">
       <c r="A40" s="1" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B40" s="3" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
   </sheetData>

</xml_diff>